<commit_message>
Updated certificate number format and added Valid for Employment Group field
- Changed certificate number format to DSYS/Game Code/Age Group Code/000001
- Added 'Valid for Employment Group' column to Excel template
- Updated bulk upload service to handle new certificate format and employment group field
- Added SAML authentication support
- Various UI and route improvements

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/templates/bulk-upload-template.xlsx
+++ b/backend/templates/bulk-upload-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Certificates" sheetId="1" r:id="rId1"/>
+    <sheet name="Athletes" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,56 +397,78 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
+  <cols>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="31.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+    <col min="11" max="11" width="27.83203125" customWidth="1"/>
+    <col min="12" max="12" width="25.83203125" customWidth="1"/>
+    <col min="13" max="13" width="21.83203125" customWidth="1"/>
+    <col min="14" max="14" width="50.83203125" customWidth="1"/>
+    <col min="15" max="15" width="19.83203125" customWidth="1"/>
+    <col min="16" max="16" width="28.83203125" customWidth="1"/>
+    <col min="17" max="17" width="17.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Name</v>
+        <v>Name of the Sports Person</v>
       </c>
       <c r="B1" t="str">
-        <v>Father Name</v>
+        <v>Father's Name / Spouse's Name</v>
       </c>
       <c r="C1" t="str">
-        <v>DOB</v>
+        <v>Date of Birth</v>
       </c>
       <c r="D1" t="str">
-        <v>District</v>
+        <v>Resident of District</v>
       </c>
       <c r="E1" t="str">
-        <v>Game Name</v>
+        <v>Representing (District/Division/State/Country)</v>
       </c>
       <c r="F1" t="str">
-        <v>Competition Period</v>
+        <v>Name of the Game</v>
       </c>
       <c r="G1" t="str">
-        <v>Competition Name</v>
+        <v>Game Code</v>
       </c>
       <c r="H1" t="str">
-        <v>Competition Held At</v>
+        <v>Age Group Code</v>
       </c>
       <c r="I1" t="str">
-        <v>Competition Level</v>
+        <v>Gender Code</v>
       </c>
       <c r="J1" t="str">
-        <v>Certificate No</v>
+        <v>Name of the Competition</v>
       </c>
       <c r="K1" t="str">
-        <v>Representing District</v>
+        <v>Period of Completion FROM</v>
       </c>
       <c r="L1" t="str">
-        <v>Division/State/Country</v>
+        <v>Period of Completion TO</v>
       </c>
       <c r="M1" t="str">
+        <v>Competition Held at</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Competition Level (State/National/International)</v>
+      </c>
+      <c r="O1" t="str">
         <v>Position Obtained</v>
       </c>
-      <c r="N1" t="str">
-        <v>Valid For Employment Group</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Applicable Govt Resolutions</v>
-      </c>
       <c r="P1" t="str">
-        <v>Email</v>
+        <v>Valid for Employment Group</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Certificate No.</v>
       </c>
     </row>
     <row r="2">
@@ -454,54 +476,57 @@
         <v>John Doe</v>
       </c>
       <c r="B2" t="str">
-        <v>James Doe</v>
+        <v>Father Name</v>
       </c>
       <c r="C2" t="str">
-        <v>01/01/1990</v>
+        <v>01-01-2000</v>
       </c>
       <c r="D2" t="str">
         <v>Mumbai</v>
       </c>
       <c r="E2" t="str">
-        <v>Kho Kho</v>
+        <v>Maharashtra</v>
       </c>
       <c r="F2" t="str">
-        <v>01/01/2024 - 05/01/2024</v>
+        <v>Cricket</v>
       </c>
       <c r="G2" t="str">
-        <v>National Championship</v>
+        <v>CRI</v>
       </c>
       <c r="H2" t="str">
-        <v>Mumbai Stadium</v>
+        <v>U19</v>
       </c>
       <c r="I2" t="str">
-        <v>National</v>
+        <v>M</v>
       </c>
       <c r="J2" t="str">
-        <v>CERT-001</v>
+        <v>State Championship</v>
       </c>
       <c r="K2" t="str">
+        <v>01-01-2025</v>
+      </c>
+      <c r="L2" t="str">
+        <v>05-01-2025</v>
+      </c>
+      <c r="M2" t="str">
         <v>Mumbai</v>
       </c>
-      <c r="L2" t="str">
-        <v>Maharashtra</v>
-      </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
+        <v>State</v>
+      </c>
+      <c r="O2" t="str">
         <v>1st</v>
       </c>
-      <c r="N2" t="str">
+      <c r="P2" t="str">
         <v>Group A</v>
       </c>
-      <c r="O2" t="str">
-        <v>GR-123/2024</v>
-      </c>
-      <c r="P2" t="str">
-        <v>john.doe@example.com</v>
+      <c r="Q2" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Changed Period of Completion to Period of Competition in Excel template
🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/templates/bulk-upload-template.xlsx
+++ b/backend/templates/bulk-upload-template.xlsx
@@ -409,8 +409,8 @@
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
     <col min="9" max="9" width="15.83203125" customWidth="1"/>
     <col min="10" max="10" width="25.83203125" customWidth="1"/>
-    <col min="11" max="11" width="27.83203125" customWidth="1"/>
-    <col min="12" max="12" width="25.83203125" customWidth="1"/>
+    <col min="11" max="11" width="28.83203125" customWidth="1"/>
+    <col min="12" max="12" width="26.83203125" customWidth="1"/>
     <col min="13" max="13" width="21.83203125" customWidth="1"/>
     <col min="14" max="14" width="50.83203125" customWidth="1"/>
     <col min="15" max="15" width="19.83203125" customWidth="1"/>
@@ -450,10 +450,10 @@
         <v>Name of the Competition</v>
       </c>
       <c r="K1" t="str">
-        <v>Period of Completion FROM</v>
+        <v>Period of Competition FROM</v>
       </c>
       <c r="L1" t="str">
-        <v>Period of Completion TO</v>
+        <v>Period of Competition TO</v>
       </c>
       <c r="M1" t="str">
         <v>Competition Held at</v>

</xml_diff>